<commit_message>
Correccion y Deep Research
</commit_message>
<xml_diff>
--- a/Análisis Paramétrico de Figuras - Conexiones de Acero.xlsx
+++ b/Análisis Paramétrico de Figuras - Conexiones de Acero.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yamip\Documents\TESINA\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89756365-6C0A-488F-BA55-E08E3C03338E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="4320" yWindow="825" windowWidth="22935" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Análisis Paramétrico de Figuras" sheetId="1" r:id="rId5"/>
+    <sheet name="Análisis Paramétrico de Figuras" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -31,9 +40,6 @@
     <t>010_Impacto del confinamiento por estribos en la resistencia al cono de concreto en tension.</t>
   </si>
   <si>
-    <t>Evalúa la variable de refuerzo transversal (estribos) en el pedestal y su influencia directa en la capacidad teórica del grupo de anclas ante fuerzas de extracción pura, mitigando la falla frágil del concreto.</t>
-  </si>
-  <si>
     <t>El confinamiento efectivo alrededor de las anclas restringe el desarrollo tridimensional del cono de falla. Esto incrementa significativamente la ductilidad local, permitiendo que la falla sea gobernada por la fluencia del acero del ancla en lugar del desprendimiento prematuro del concreto.</t>
   </si>
   <si>
@@ -43,9 +49,6 @@
     <t>011_Requisitos de distancia minima al borde libre impacto normativo del cambio para anclas.</t>
   </si>
   <si>
-    <t>Modela la sensibilidad de la capacidad de anclaje frente a la variable geométrica c_{a1} (distancia al borde libre), evaluando el umbral donde el desprendimiento lateral (side-face blowout) gobierna el diseño.</t>
-  </si>
-  <si>
     <t>Se evidencia una penalización severa en la resistencia disponible a medida que los anclajes se acercan a los bordes del pedestal. Los datos demuestran que las distancias mínimas no son solo tolerancias constructivas, sino límites mecánicos para evitar fallas por tracción diagonal en el recubrimiento.</t>
   </si>
   <si>
@@ -55,9 +58,6 @@
     <t>013_Mapa de calor_Incremento de resistencia al cono de tension-NTC-2023 vs NTC-2017.</t>
   </si>
   <si>
-    <t>Cuantifica la divergencia matemática entre las formulaciones de la NTC-2017 y la NTC-2023 para la resistencia a la tensión (N_{cbg}), mapeando variaciones según la profundidad de embebido (h_{ef}) y la separación entre anclas (s).</t>
-  </si>
-  <si>
     <t>Comparativa Normativa: Revela zonas geométricas específicas donde la NTC-2023 resulta ser más conservadora. El incremento o decremento en la resistencia calculada refleja una calibración más estricta en los factores de grupo y excentricidad, penalizando configuraciones que antes se consideraban holgadas.</t>
   </si>
   <si>
@@ -70,68 +70,158 @@
     <t>Contrasta la capacidad de carga lateral (R_v) soportada por los anclajes antes de la falla por cortante en el concreto, analizando cómo el cambio normativo altera las curvas de resistencia esperada frente al cortante basal.</t>
   </si>
   <si>
-    <t>Comparativa Normativa: El salto a la NTC-2023 modifica la envolvente de falla por cortante hacia el borde libre. La tendencia indica que la nueva normativa ajusta la contribución de anclajes múltiples bajo carga lateral, reduciendo la capacidad predictiva en configuraciones con anclas frontales y traseras que no distribuyen el cortante uniformemente.</t>
-  </si>
-  <si>
-    <t>Dictamina la viabilidad de transmitir cortante basal severo (ej. en marcos rígidos) puramente a través de anclas. Demuestra cuándo es imperativo migrar el diseño hacia el uso de llaves de cortante (shear lugs) o depender de la fricción bajo las normas vigentes.</t>
+    <t>Modela la sensibilidad de la capacidad de anclaje frente a la variable geométrica c_{min} (distancia al borde libre), evaluando el umbral donde el desprendimiento lateral (side-face blowout) gobierna el diseño.</t>
+  </si>
+  <si>
+    <t>Cuantifica la divergencia matemática entre las formulaciones de la NTC-2017 y la NTC-2023 para la resistencia a la tensión, mapeando variaciones según la profundidad de embebido (h_{ef}) y la separación entre anclas (s).</t>
+  </si>
+  <si>
+    <t>Evalúa la variable de refuerzo transversal (estribos) en el pedestal y su influencia directa en la capacidad del grupo de anclas ante fuerzas de extracción pura, mitigando la falla frágil del concreto.</t>
+  </si>
+  <si>
+    <t>La NTC 2023 reduce de forma matemática la resistencia de diseño en comparación con la NTC 2017 para configuraciones de anclas en fila. Debido a que la nueva norma reconoce que las anclas más cercanas al borde libre absorben la mayor parte del cortante, evitando que las filas posteriores colaboren de manera uniforme antes de que ocurra la fractura del concreto.</t>
+  </si>
+  <si>
+    <t>Dictamina la eficiencia estructural ante cortante basal. La NTC 2023 penaliza severamente el efecto de grupo en filas alineadas a la carga, volviendo ineficaz esta solución. Esto exige optimizar el diseño priorizando arreglos ortogonales al empuje, evitando saturar la conexión con anclajes inoperantes antes de la fractura del concreto frontal.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFEBFFEB"/>
+    </mruColors>
+  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -321,102 +411,114 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="50.140625" customWidth="1"/>
+    <col min="4" max="4" width="63.5703125" customWidth="1"/>
+    <col min="5" max="5" width="63.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:5" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="C3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
+    <row r="4" spans="1:5" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="C4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="E4" s="11" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1">
-        <v>3.0</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="1" t="s">
+    <row r="5" spans="1:5" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>16</v>
+      <c r="D5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1">
-        <v>4.0</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>20</v>
-      </c>
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="1"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>